<commit_message>
Sync solarheatingsecond: tank cost correction factor, report center, combined-mode recommendation fix
- Tank unit-cost model y=c+a*V^b with correction factor k inputs (seasonal k=1.1), recorded in reports
- GUI: /reports static links + Report Center sidebar panel
- Fix: combined-mode recommendation panels now stay on full-grid basis instead of being overwritten by Step-2 tank study
- Add grid_comparison.py, heating_load_sensitivity.py, run_gui.bat, analysis docs and code backups
</commit_message>
<xml_diff>
--- a/design_inputs.xlsx
+++ b/design_inputs.xlsx
@@ -413,311 +413,529 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AK2"/>
+  <dimension ref="A1:BK2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>project_name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>tank_max_temp</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>small_delta_t_tank_min_temp</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>large_delta_t_tank_min_temp</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>initial_tank_temp</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>heating_supply_temp</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>heating_delta_t</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>solar_collector_delta_t</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>collector_flow_lph_per_m2</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>collector_delta_t_min_c</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>collector_delta_t_max_c</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>direct_solar_delivery_margin_c</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
         <is>
           <t>short_term_loss</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>seasonal_loss</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>short_term_ratio</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>seasonal_ratio</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>short_term_preset</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>seasonal_preset</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>short_term_tank_height_m</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>seasonal_tank_height_m</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>short_term_static_mixing_coeff</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>seasonal_static_mixing_coeff</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>short_term_charge_mixing_coeff</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>seasonal_charge_mixing_coeff</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>short_term_discharge_mixing_coeff</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>seasonal_discharge_mixing_coeff</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
         <is>
           <t>collector_cost_per_m2</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>project_lifetime_years</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>electricity_price</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>electric_boiler_efficiency</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>heat_pump_cop</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>short_term_cost_coeff</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>short_term_cost_exponent</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>seasonal_cost_coeff</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>seasonal_cost_exponent</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
+        <is>
+          <t>short_term_cost_asymptote</t>
+        </is>
+      </c>
+      <c r="AG1" t="inlineStr">
+        <is>
+          <t>short_term_cost_scale</t>
+        </is>
+      </c>
+      <c r="AH1" t="inlineStr">
+        <is>
+          <t>short_term_cost_power</t>
+        </is>
+      </c>
+      <c r="AI1" t="inlineStr">
+        <is>
+          <t>seasonal_cost_asymptote</t>
+        </is>
+      </c>
+      <c r="AJ1" t="inlineStr">
+        <is>
+          <t>seasonal_cost_scale</t>
+        </is>
+      </c>
+      <c r="AK1" t="inlineStr">
+        <is>
+          <t>seasonal_cost_power</t>
+        </is>
+      </c>
+      <c r="AL1" t="inlineStr">
+        <is>
+          <t>short_term_cost_correction_factor</t>
+        </is>
+      </c>
+      <c r="AM1" t="inlineStr">
+        <is>
+          <t>seasonal_cost_correction_factor</t>
+        </is>
+      </c>
+      <c r="AN1" t="inlineStr">
         <is>
           <t>sizing_mode</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="AO1" t="inlineStr">
         <is>
           <t>short_collector_min_size</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="AP1" t="inlineStr">
         <is>
           <t>short_collector_max_size</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="AQ1" t="inlineStr">
         <is>
           <t>short_collector_count</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="AR1" t="inlineStr">
         <is>
           <t>short_tank_min_size</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AS1" t="inlineStr">
         <is>
           <t>short_tank_max_size</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AT1" t="inlineStr">
         <is>
           <t>short_tank_count</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AU1" t="inlineStr">
         <is>
           <t>long_collector_min_size</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AV1" t="inlineStr">
         <is>
           <t>long_collector_max_size</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AW1" t="inlineStr">
         <is>
           <t>long_collector_count</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AX1" t="inlineStr">
         <is>
           <t>long_tank_min_size</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AY1" t="inlineStr">
         <is>
           <t>long_tank_max_size</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AZ1" t="inlineStr">
         <is>
           <t>long_tank_count</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="BA1" t="inlineStr">
         <is>
           <t>collector_type</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="BB1" t="inlineStr">
         <is>
           <t>eta0</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="BC1" t="inlineStr">
         <is>
           <t>a1</t>
         </is>
       </c>
-      <c r="AK1" t="inlineStr">
+      <c r="BD1" t="inlineStr">
         <is>
           <t>a2</t>
+        </is>
+      </c>
+      <c r="BE1" t="inlineStr">
+        <is>
+          <t>collector_soiling_factor</t>
+        </is>
+      </c>
+      <c r="BF1" t="inlineStr">
+        <is>
+          <t>optimization_selection_mode</t>
+        </is>
+      </c>
+      <c r="BG1" t="inlineStr">
+        <is>
+          <t>optimization_cost_tolerance_pct</t>
+        </is>
+      </c>
+      <c r="BH1" t="inlineStr">
+        <is>
+          <t>optimization_min_solar_coverage_pct</t>
+        </is>
+      </c>
+      <c r="BI1" t="inlineStr">
+        <is>
+          <t>optimization_auto_refine_search</t>
+        </is>
+      </c>
+      <c r="BJ1" t="inlineStr">
+        <is>
+          <t>optimization_refine_span_pct</t>
+        </is>
+      </c>
+      <c r="BK1" t="inlineStr">
+        <is>
+          <t>selected_scenarios</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>测试clzk</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
         <v>80</v>
       </c>
-      <c r="B2" t="n">
+      <c r="C2" t="n">
         <v>35</v>
       </c>
-      <c r="C2" t="n">
+      <c r="D2" t="n">
         <v>8</v>
       </c>
-      <c r="D2" t="n">
-        <v>35</v>
-      </c>
       <c r="E2" t="n">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="F2" t="n">
-        <v>10</v>
+        <v>46</v>
       </c>
       <c r="G2" t="n">
         <v>10</v>
       </c>
       <c r="H2" t="n">
+        <v>20</v>
+      </c>
+      <c r="I2" t="n">
+        <v>25</v>
+      </c>
+      <c r="J2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K2" t="n">
+        <v>20</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" t="n">
+        <v>5</v>
+      </c>
+      <c r="N2" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="O2" t="n">
+        <v>50</v>
+      </c>
+      <c r="P2" t="n">
+        <v>2000</v>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>Poor</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="S2" t="n">
+        <v>6</v>
+      </c>
+      <c r="T2" t="n">
+        <v>10</v>
+      </c>
+      <c r="U2" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="V2" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="W2" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="X2" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>0.018</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>2150</v>
+      </c>
+      <c r="AB2" t="n">
+        <v>20</v>
+      </c>
+      <c r="AC2" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="AD2" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="AE2" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="AF2" t="n">
+        <v>585.8</v>
+      </c>
+      <c r="AG2" t="n">
+        <v>18470</v>
+      </c>
+      <c r="AH2" t="n">
+        <v>-0.576</v>
+      </c>
+      <c r="AI2" t="n">
+        <v>196.3</v>
+      </c>
+      <c r="AJ2" t="n">
+        <v>1313000</v>
+      </c>
+      <c r="AK2" t="n">
+        <v>-0.9350000000000001</v>
+      </c>
+      <c r="AL2" t="n">
         <v>1</v>
       </c>
-      <c r="I2" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="J2" t="n">
-        <v>200</v>
-      </c>
-      <c r="K2" t="n">
-        <v>2000</v>
-      </c>
-      <c r="L2" t="n">
-        <v>800</v>
-      </c>
-      <c r="M2" t="n">
-        <v>25</v>
-      </c>
-      <c r="N2" t="n">
-        <v>0.12</v>
-      </c>
-      <c r="O2" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="P2" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>1400</v>
-      </c>
-      <c r="R2" t="n">
-        <v>0.78</v>
-      </c>
-      <c r="S2" t="n">
-        <v>900</v>
-      </c>
-      <c r="T2" t="n">
-        <v>0.82</v>
-      </c>
-      <c r="U2" t="inlineStr">
+      <c r="AM2" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="AN2" t="inlineStr">
         <is>
           <t>Auto Generate</t>
         </is>
       </c>
-      <c r="V2" t="n">
-        <v>100</v>
-      </c>
-      <c r="W2" t="n">
+      <c r="AO2" t="n">
+        <v>5000</v>
+      </c>
+      <c r="AP2" t="n">
         <v>50000</v>
       </c>
-      <c r="X2" t="n">
-        <v>10</v>
-      </c>
-      <c r="Y2" t="n">
-        <v>10</v>
-      </c>
-      <c r="Z2" t="n">
-        <v>6000</v>
-      </c>
-      <c r="AA2" t="n">
-        <v>10</v>
-      </c>
-      <c r="AB2" t="n">
-        <v>200</v>
-      </c>
-      <c r="AC2" t="n">
+      <c r="AQ2" t="n">
+        <v>20</v>
+      </c>
+      <c r="AR2" t="n">
+        <v>1000</v>
+      </c>
+      <c r="AS2" t="n">
+        <v>10000</v>
+      </c>
+      <c r="AT2" t="n">
+        <v>20</v>
+      </c>
+      <c r="AU2" t="n">
+        <v>5000</v>
+      </c>
+      <c r="AV2" t="n">
         <v>50000</v>
       </c>
-      <c r="AD2" t="n">
-        <v>10</v>
-      </c>
-      <c r="AE2" t="n">
-        <v>100</v>
-      </c>
-      <c r="AF2" t="n">
+      <c r="AW2" t="n">
+        <v>20</v>
+      </c>
+      <c r="AX2" t="n">
+        <v>10000</v>
+      </c>
+      <c r="AY2" t="n">
         <v>100000</v>
       </c>
-      <c r="AG2" t="n">
-        <v>10</v>
-      </c>
-      <c r="AH2" t="inlineStr">
+      <c r="AZ2" t="n">
+        <v>20</v>
+      </c>
+      <c r="BA2" t="inlineStr">
         <is>
           <t>Evacuated Tube</t>
         </is>
       </c>
-      <c r="AI2" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="AJ2" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="AK2" t="n">
-        <v>0.005</v>
+      <c r="BB2" t="n">
+        <v>0.464</v>
+      </c>
+      <c r="BC2" t="n">
+        <v>1.141</v>
+      </c>
+      <c r="BD2" t="n">
+        <v>0.0028</v>
+      </c>
+      <c r="BE2" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="BF2" t="inlineStr">
+        <is>
+          <t>compact_near_optimal</t>
+        </is>
+      </c>
+      <c r="BG2" t="n">
+        <v>5</v>
+      </c>
+      <c r="BH2" t="n">
+        <v>60</v>
+      </c>
+      <c r="BI2" t="b">
+        <v>0</v>
+      </c>
+      <c r="BJ2" t="n">
+        <v>35</v>
+      </c>
+      <c r="BK2" t="inlineStr">
+        <is>
+          <t>seasonal_boiler</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>